<commit_message>
feat(audit): implement closeout lifecycle, multi-course support, and site library Add audit phase schema and migration with lead faculty fields in Setup. Introduce course defaults, courseId, and course-aware semester/faculty file naming. Add program clinical site library integration across Setup and Advanced Configuration. Ship Audit tab with attestation workflow, audit PDF export, and SHA-256 snapshot hashing. Enforce read-only guards during export/lock phases and record makeup provenance when slots are applied. Add audit snapshot/export tests and update implementation documentation.
</commit_message>
<xml_diff>
--- a/protypes/2026 Spring - 15 & 15P 1-23-26.xlsx
+++ b/protypes/2026 Spring - 15 & 15P 1-23-26.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6f59b093a0d7fd64/Desktop/REGN 15P Sim and Clinical Tracker/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6f59b093a0d7fd64/Desktop/REGN 15P Sim and Clinical Tracker/protypes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="26" documentId="8_{87988D37-CE1A-4900-97F1-6C2FC5B82D7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B9D4D2FB-DB49-42CF-977A-AA1220D414C3}"/>
+  <xr:revisionPtr revIDLastSave="27" documentId="8_{87988D37-CE1A-4900-97F1-6C2FC5B82D7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{50DDC60F-9BE0-4E96-9F30-6B7937E47B15}"/>
   <bookViews>
     <workbookView xWindow="-25710" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{080C685D-B7D8-4AC0-9B4D-985EAD6D7FC2}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="580" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="581" uniqueCount="68">
   <si>
     <t>Simulation and Clinical Schedule</t>
   </si>
@@ -239,6 +239,9 @@
   </si>
   <si>
     <t>Faculty 1</t>
+  </si>
+  <si>
+    <t>Orient-SE</t>
   </si>
 </sst>
 </file>
@@ -606,16 +609,16 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -636,6 +639,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -968,13 +975,13 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:44" x14ac:dyDescent="0.25">
-      <c r="A2" s="73" t="s">
+      <c r="A2" s="71" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="73"/>
-      <c r="C2" s="73"/>
-      <c r="D2" s="73"/>
-      <c r="E2" s="73"/>
+      <c r="B2" s="71"/>
+      <c r="C2" s="71"/>
+      <c r="D2" s="71"/>
+      <c r="E2" s="71"/>
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
       <c r="H2" s="1"/>
@@ -1011,11 +1018,11 @@
       <c r="AM2" s="1"/>
       <c r="AN2" s="1"/>
       <c r="AO2" s="1"/>
-      <c r="AP2" s="74" t="s">
+      <c r="AP2" s="72" t="s">
         <v>1</v>
       </c>
-      <c r="AQ2" s="74"/>
-      <c r="AR2" s="74"/>
+      <c r="AQ2" s="72"/>
+      <c r="AR2" s="72"/>
     </row>
     <row r="3" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A3" s="2"/>
@@ -1155,74 +1162,74 @@
         <v>1</v>
       </c>
       <c r="G4" s="7"/>
-      <c r="H4" s="71">
+      <c r="H4" s="73">
         <v>2</v>
       </c>
-      <c r="I4" s="72"/>
-      <c r="J4" s="71">
+      <c r="I4" s="74"/>
+      <c r="J4" s="73">
         <v>3</v>
       </c>
-      <c r="K4" s="72"/>
-      <c r="L4" s="71">
+      <c r="K4" s="74"/>
+      <c r="L4" s="73">
         <v>4</v>
       </c>
-      <c r="M4" s="72"/>
-      <c r="N4" s="71">
+      <c r="M4" s="74"/>
+      <c r="N4" s="73">
         <v>5</v>
       </c>
       <c r="O4" s="75"/>
-      <c r="P4" s="71">
+      <c r="P4" s="73">
         <v>6</v>
       </c>
-      <c r="Q4" s="72"/>
-      <c r="R4" s="71">
+      <c r="Q4" s="74"/>
+      <c r="R4" s="73">
         <v>7</v>
       </c>
-      <c r="S4" s="72"/>
-      <c r="T4" s="71">
+      <c r="S4" s="74"/>
+      <c r="T4" s="73">
         <v>8</v>
       </c>
-      <c r="U4" s="72"/>
-      <c r="V4" s="71">
+      <c r="U4" s="74"/>
+      <c r="V4" s="73">
         <v>9</v>
       </c>
-      <c r="W4" s="72"/>
-      <c r="X4" s="71">
+      <c r="W4" s="74"/>
+      <c r="X4" s="73">
         <v>10</v>
       </c>
-      <c r="Y4" s="72"/>
-      <c r="Z4" s="71">
+      <c r="Y4" s="74"/>
+      <c r="Z4" s="73">
         <v>11</v>
       </c>
-      <c r="AA4" s="72"/>
-      <c r="AB4" s="71">
+      <c r="AA4" s="74"/>
+      <c r="AB4" s="73">
         <v>12</v>
       </c>
-      <c r="AC4" s="72"/>
-      <c r="AD4" s="71">
+      <c r="AC4" s="74"/>
+      <c r="AD4" s="73">
         <v>13</v>
       </c>
-      <c r="AE4" s="72"/>
-      <c r="AF4" s="71">
+      <c r="AE4" s="74"/>
+      <c r="AF4" s="73">
         <v>14</v>
       </c>
-      <c r="AG4" s="72"/>
-      <c r="AH4" s="71">
+      <c r="AG4" s="74"/>
+      <c r="AH4" s="73">
         <v>15</v>
       </c>
-      <c r="AI4" s="72"/>
-      <c r="AJ4" s="71">
+      <c r="AI4" s="74"/>
+      <c r="AJ4" s="73">
         <v>16</v>
       </c>
-      <c r="AK4" s="72"/>
-      <c r="AL4" s="71">
+      <c r="AK4" s="74"/>
+      <c r="AL4" s="73">
         <v>17</v>
       </c>
-      <c r="AM4" s="72"/>
-      <c r="AN4" s="71">
-        <v>18</v>
-      </c>
-      <c r="AO4" s="74"/>
+      <c r="AM4" s="74"/>
+      <c r="AN4" s="73">
+        <v>18</v>
+      </c>
+      <c r="AO4" s="72"/>
       <c r="AP4" s="6"/>
       <c r="AQ4" s="2"/>
       <c r="AR4" s="2"/>
@@ -2149,7 +2156,9 @@
       </c>
       <c r="F15" s="44"/>
       <c r="G15" s="49"/>
-      <c r="H15" s="18"/>
+      <c r="H15" s="18" t="s">
+        <v>67</v>
+      </c>
       <c r="I15" s="17"/>
       <c r="J15" s="44"/>
       <c r="K15" s="17"/>
@@ -4163,6 +4172,9 @@
     </row>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="AD4:AE4"/>
+    <mergeCell ref="AF4:AG4"/>
+    <mergeCell ref="AH4:AI4"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="AP2:AR2"/>
     <mergeCell ref="H4:I4"/>
@@ -4179,27 +4191,24 @@
     <mergeCell ref="X4:Y4"/>
     <mergeCell ref="Z4:AA4"/>
     <mergeCell ref="AB4:AC4"/>
-    <mergeCell ref="AD4:AE4"/>
-    <mergeCell ref="AF4:AG4"/>
-    <mergeCell ref="AH4:AI4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4365,18 +4374,18 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{916F09E3-27E3-460A-9F8E-1C97730F458C}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{96E3F7F7-3DDE-4B82-A6A3-D25E362514B5}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{96E3F7F7-3DDE-4B82-A6A3-D25E362514B5}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{916F09E3-27E3-460A-9F8E-1C97730F458C}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>